<commit_message>
Add Supabase connection and environment variables
</commit_message>
<xml_diff>
--- a/Template/planilla_financiera_2024_2025.xlsx
+++ b/Template/planilla_financiera_2024_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jspez\Documents\Proyectos\Emprendimiento\FinanceReports\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7493CB24-722F-4835-B696-7086C6C9CB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5612858A-41F0-4617-B6F8-DA26824713F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="transactions_finance" sheetId="1" r:id="rId1"/>
@@ -2957,6 +2957,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M301"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>